<commit_message>
refactor: hapus kolom departemen dari template excel dan perketat validasi impor via modal error
</commit_message>
<xml_diff>
--- a/public/templates/Template_Penyesuaian_Persediaan.xlsx
+++ b/public/templates/Template_Penyesuaian_Persediaan.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -492,8 +492,7 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="33" customHeight="1">
@@ -534,11 +533,6 @@
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
-          <t>Nama Dept Barang</t>
-        </is>
-      </c>
-      <c r="I1" s="3" t="inlineStr">
-        <is>
           <t>Keterangan</t>
         </is>
       </c>
@@ -575,8 +569,7 @@
           <t>Penambahan</t>
         </is>
       </c>
-      <c r="H2" s="6" t="n"/>
-      <c r="I2" s="6" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>Penyesuaian hasil stok opname fisik</t>
         </is>
@@ -614,8 +607,7 @@
           <t>Pengurangan</t>
         </is>
       </c>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="6" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Batang bengkok / cacat pabrik</t>
         </is>
@@ -653,8 +645,7 @@
           <t>Penambahan</t>
         </is>
       </c>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>Selisih lebih barang masuk</t>
         </is>
@@ -671,13 +662,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="140" customWidth="1" min="4" max="4"/>
+    <col width="130" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -734,7 +725,7 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>Isi kolom dengan nama barang, tapi kecocokan dengan penamaan dalam accurate Online akan di abaikan</t>
+          <t>Isi kolom dengan nama barang. Sistem menggunakan nama ini sebagai alternatif pencocokan jika kode tidak diisi.</t>
         </is>
       </c>
     </row>
@@ -756,7 +747,7 @@
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>Isi dengan kode barang, kolom ini harus tepat kode nya dengan accurate online. Akan jadi acuan apakah barang ada atau tidak dalam database</t>
+          <t>Isi dengan kode barang/SKU. Kolom ini menjadi acuan utama pencocokan barang dalam database.</t>
         </is>
       </c>
     </row>
@@ -778,7 +769,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Isi dengan nama unit barang, kolom ini harus tepat nama unit nya dengan accurate online. Akan jadi acuan apakah barang ada atau tidak dalam database.</t>
+          <t>Isi dengan nama unit/satuan barang (misal: SAK, BTG, PCS). Jika kosong, sistem otomatis memakai satuan default barang.</t>
         </is>
       </c>
     </row>
@@ -800,7 +791,7 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>Isi dengan kuantitas barang</t>
+          <t>Isi dengan kuantitas penyesuaian barang (harus berupa angka lebih dari 0).</t>
         </is>
       </c>
     </row>
@@ -822,7 +813,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Isi dengan biaya satuan barang</t>
+          <t>Isi dengan biaya satuan barang (HPP). Jika kosong, sistem otomatis memakai nilai biaya satuan dari database.</t>
         </is>
       </c>
     </row>
@@ -844,7 +835,7 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>Isi kolom dengan nama gudang, kolom ini harus tepat nama gudang nya dengan accurate online.</t>
+          <t>Isi dengan nama gudang barang (misal: Toko Utama). Kolom ini harus tepat namanya.</t>
         </is>
       </c>
     </row>
@@ -859,17 +850,21 @@
           <t>Wajib</t>
         </is>
       </c>
-      <c r="C10" s="9" t="n"/>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Isi dengan Penambahan / Pengurangan / Atur Stok</t>
+          <t>Isi dengan "Penambahan" atau "Pengurangan".</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Nama Dept Barang</t>
+          <t>Keterangan</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -879,34 +874,12 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>240</t>
+          <t>255</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Nama departemen pada rincian barang</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Keterangan</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Tidak Wajib</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>Catatan atau keterangan penyesuaian untuk baris barang tersebut</t>
+          <t>Catatan alasan atau keterangan penyesuaian pada baris barang tersebut.</t>
         </is>
       </c>
     </row>

</xml_diff>